<commit_message>
Ajout colonnes contact et message email dans clients.xlsx
Nouvelles colonnes : Nom interlocuteur, Poste/Fonction, Email interlocuteur,
Message email (template personnalisé par client). Emails préremplis pour DMD et ORTEC.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/clients.xlsx
+++ b/clients.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Clients'!$A$1:$L$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Clients'!$A$1:$O$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -60,8 +60,9 @@
       <name val="Arial"/>
       <sz val="11"/>
     </font>
+    <font/>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -83,8 +84,13 @@
         <fgColor rgb="00E8F5E9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF8E1"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -106,11 +112,12 @@
         <color rgb="00D0D0D0"/>
       </bottom>
     </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -132,6 +139,10 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -497,7 +508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:T6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -509,9 +520,12 @@
     <col width="20" customWidth="1" min="7" max="7"/>
     <col width="28" customWidth="1" min="8" max="8"/>
     <col width="30" customWidth="1" min="9" max="9"/>
-    <col width="25" customWidth="1" min="10" max="10"/>
-    <col width="15" customWidth="1" min="11" max="11"/>
-    <col width="45" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="12" max="12"/>
+    <col width="55" customWidth="1" min="13" max="13"/>
+    <col width="15" customWidth="1" min="14" max="14"/>
+    <col width="45" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="35" customHeight="1">
@@ -562,19 +576,39 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Interlocuteur / Contact</t>
+          <t>Nom interlocuteur</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>Poste / Fonction</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Email interlocuteur</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Message email</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t>Statut</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Fichier PPTX genere</t>
         </is>
       </c>
+      <c r="P1" s="9" t="n"/>
+      <c r="Q1" s="9" t="n"/>
+      <c r="R1" s="9" t="n"/>
+      <c r="S1" s="9" t="n"/>
+      <c r="T1" s="9" t="n"/>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -622,21 +656,43 @@
           <t>dashboard  Conwise Fleet manager pour DMD groupe.png</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>Fleet Manager DMD</t>
-        </is>
-      </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Fleet Manager</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="10" t="inlineStr">
+        <is>
+          <t>Bonjour [Prenom],
+Suite a notre echange, j ai le plaisir de vous adresser notre proposition pour la gestion et le convoyage de la flotte du Groupe DMD.
+Vous trouverez en piece jointe une presentation detaillee de nos services adaptes a votre organisation multi-sites.
+Points cles de notre offre :
+- Convoyeurs professionnels certifies et assures
+- Portail de gestion dedie Groupe DMD sur conwise.app
+- Livraison sous 24-48h sur toute la France
+- Etat des lieux digital systematique
+Je reste a votre disposition pour organiser un echange et repondre a vos questions.
+Cordialement,
+Conwise Express</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="inlineStr">
         <is>
           <t>Fait</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>Proposition Conwise Express - Groupe DMD.pptx</t>
         </is>
       </c>
+      <c r="P2" s="9" t="n"/>
+      <c r="Q2" s="9" t="n"/>
+      <c r="R2" s="9" t="n"/>
+      <c r="S2" s="9" t="n"/>
+      <c r="T2" s="9" t="n"/>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
@@ -684,21 +740,43 @@
           <t>dashboard Fleet manager Groupe Ortec.png</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
-        <is>
-          <t>Fleet Manager ORTEC</t>
-        </is>
-      </c>
-      <c r="K3" s="3" t="inlineStr">
+      <c r="J3" s="4" t="inlineStr"/>
+      <c r="K3" s="4" t="inlineStr">
+        <is>
+          <t>Fleet Manager</t>
+        </is>
+      </c>
+      <c r="L3" s="4" t="inlineStr"/>
+      <c r="M3" s="10" t="inlineStr">
+        <is>
+          <t>Bonjour [Prenom],
+Suite a notre echange, j ai le plaisir de vous adresser notre proposition pour la prise en charge des transferts et rapatriements de la flotte du Groupe ORTEC sur vos agences en France.
+Nous accompagnons deja des groupes multi-sites de votre envergure comme Derichebourg (48 000 collaborateurs, 150 sites) sur l ensemble de leur logistique flotte.
+Notre proposition inclut :
+- Transferts inter-agences et services carrosserie
+- Portail de gestion dedie Groupe ORTEC sur conwise.app
+- Tracabilite complete et PV digitalises
+- Couverture nationale sous 24-48h
+Je reste a votre disposition pour organiser un echange.
+Cordialement,
+Conwise Express</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
         <is>
           <t>Fait</t>
         </is>
       </c>
-      <c r="L3" s="4" t="inlineStr">
+      <c r="O3" s="4" t="inlineStr">
         <is>
           <t>Proposition Conwise Express x Groupe ORTEC.pptx</t>
         </is>
       </c>
+      <c r="P3" s="9" t="n"/>
+      <c r="Q3" s="9" t="n"/>
+      <c r="R3" s="9" t="n"/>
+      <c r="S3" s="9" t="n"/>
+      <c r="T3" s="9" t="n"/>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="2" t="inlineStr"/>
@@ -715,12 +793,20 @@
       <c r="H4" s="2" t="inlineStr"/>
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr"/>
-      <c r="K4" s="5" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr"/>
+      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr"/>
+      <c r="N4" s="5" t="inlineStr">
         <is>
           <t>A faire</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr"/>
+      <c r="O4" s="2" t="inlineStr"/>
+      <c r="P4" s="9" t="n"/>
+      <c r="Q4" s="9" t="n"/>
+      <c r="R4" s="9" t="n"/>
+      <c r="S4" s="9" t="n"/>
+      <c r="T4" s="9" t="n"/>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="4" t="inlineStr"/>
@@ -737,12 +823,20 @@
       <c r="H5" s="4" t="inlineStr"/>
       <c r="I5" s="4" t="inlineStr"/>
       <c r="J5" s="4" t="inlineStr"/>
-      <c r="K5" s="6" t="inlineStr">
+      <c r="K5" s="4" t="inlineStr"/>
+      <c r="L5" s="4" t="inlineStr"/>
+      <c r="M5" s="4" t="inlineStr"/>
+      <c r="N5" s="6" t="inlineStr">
         <is>
           <t>A faire</t>
         </is>
       </c>
-      <c r="L5" s="4" t="inlineStr"/>
+      <c r="O5" s="4" t="inlineStr"/>
+      <c r="P5" s="9" t="n"/>
+      <c r="Q5" s="9" t="n"/>
+      <c r="R5" s="9" t="n"/>
+      <c r="S5" s="9" t="n"/>
+      <c r="T5" s="9" t="n"/>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="2" t="inlineStr"/>
@@ -759,15 +853,23 @@
       <c r="H6" s="2" t="inlineStr"/>
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr"/>
-      <c r="K6" s="5" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr"/>
+      <c r="L6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="inlineStr"/>
+      <c r="N6" s="5" t="inlineStr">
         <is>
           <t>A faire</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr"/>
+      <c r="O6" s="2" t="inlineStr"/>
+      <c r="P6" s="9" t="n"/>
+      <c r="Q6" s="9" t="n"/>
+      <c r="R6" s="9" t="n"/>
+      <c r="S6" s="9" t="n"/>
+      <c r="T6" s="9" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L6"/>
+  <autoFilter ref="A1:O6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -778,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="1" max="1"/>
@@ -797,7 +899,7 @@
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>1. Remplir une ligne par client dans l'onglet "Clients"</t>
+          <t>1. Remplir une ligne par client dans l'onglet Clients</t>
         </is>
       </c>
     </row>
@@ -835,14 +937,14 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">   "Lis le fichier clients.xlsx et genere la presentation</t>
+          <t xml:space="preserve">   "Lis clients.xlsx et genere la presentation + email</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">   pour le client en ligne [X] (ou tous ceux A faire)."</t>
+          <t xml:space="preserve">   pour tous les clients A faire."</t>
         </is>
       </c>
     </row>
@@ -852,14 +954,14 @@
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>5. Claude genere automatiquement le PPTX personnalise</t>
+          <t>5. Claude genere le PPTX + redige le message email personnalise</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>6. Mettre a jour le statut et le nom du fichier dans le tableau</t>
+          <t>6. Mettre a jour le statut dans le tableau</t>
         </is>
       </c>
     </row>
@@ -880,6 +982,16 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>COLONNES EMAIL : Nom interlocuteur, Poste, Email, Message email</t>
+        </is>
+      </c>
+    </row>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>